<commit_message>
#6 Peripheral added in BOM.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM-Brendon_STM32-v1.1.xlsx
+++ b/Design_Files/BOM/Client_BOM-Brendon_STM32-v1.1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\brendanbezuko-stm32pcb\Design_Files\Project Outputs for Brendon_STM32-v1.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\brendanbezuko-stm32pcb\Design_Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="174">
   <si>
     <t>#</t>
   </si>
@@ -523,13 +523,31 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Radio Module 437MHz</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t>Through Hole-2.54mm</t>
+  </si>
+  <si>
+    <t>Through Hole-1.27mm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -579,6 +597,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -600,7 +626,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -691,11 +717,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -732,20 +789,122 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1039,35 +1198,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="5" max="5" width="30" style="24" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.5703125" style="21" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="4" customWidth="1"/>
+    <col min="12" max="12" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="E1" s="22"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="G1" s="18"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+    </row>
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1078,7 +1239,7 @@
       <c r="D2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="23" t="s">
         <v>47</v>
       </c>
       <c r="F2" s="5" t="s">
@@ -1097,10 +1258,13 @@
         <v>159</v>
       </c>
       <c r="K2" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1118,7 +1282,7 @@
       <c r="F3" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="19" t="s">
         <v>99</v>
       </c>
       <c r="H3" s="7" t="s">
@@ -1130,9 +1294,12 @@
       <c r="J3" s="7">
         <v>19</v>
       </c>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L3" s="7"/>
+    </row>
+    <row r="4" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B34" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1150,7 +1317,7 @@
       <c r="F4" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="20" t="s">
         <v>100</v>
       </c>
       <c r="H4" s="9" t="s">
@@ -1162,9 +1329,12 @@
       <c r="J4" s="9">
         <v>2</v>
       </c>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1182,7 +1352,7 @@
       <c r="F5" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="19" t="s">
         <v>101</v>
       </c>
       <c r="H5" s="7" t="s">
@@ -1194,9 +1364,12 @@
       <c r="J5" s="7">
         <v>1</v>
       </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L5" s="7"/>
+    </row>
+    <row r="6" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1214,7 +1387,7 @@
       <c r="F6" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="20" t="s">
         <v>102</v>
       </c>
       <c r="H6" s="9" t="s">
@@ -1226,9 +1399,12 @@
       <c r="J6" s="9">
         <v>3</v>
       </c>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L6" s="9"/>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1246,7 +1422,7 @@
       <c r="F7" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="19" t="s">
         <v>103</v>
       </c>
       <c r="H7" s="7" t="s">
@@ -1258,9 +1434,12 @@
       <c r="J7" s="7">
         <v>4</v>
       </c>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K7" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L7" s="7"/>
+    </row>
+    <row r="8" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1278,21 +1457,24 @@
       <c r="F8" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="20" t="s">
         <v>104</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L8" s="9"/>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1301,24 +1483,27 @@
       <c r="C9" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="8"/>
       <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
+      <c r="G9" s="19"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="J9" s="16">
+      <c r="I9" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="J9" s="15">
         <v>3</v>
       </c>
-      <c r="K9" s="16" t="s">
+      <c r="K9" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L9" s="15" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1333,22 +1518,27 @@
       <c r="E10" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="10">
+      <c r="F10" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="G10" s="20">
         <v>22232021</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J10" s="9">
         <v>4</v>
       </c>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K10" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1363,22 +1553,27 @@
       <c r="E11" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8" t="s">
+      <c r="F11" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="G11" s="19" t="s">
         <v>105</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="I11" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K11" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L11" s="7"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1393,22 +1588,27 @@
       <c r="E12" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10">
+      <c r="F12" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="G12" s="20">
         <v>22232041</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K12" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1426,21 +1626,24 @@
       <c r="F13" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="19" t="s">
         <v>106</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K13" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L13" s="7"/>
+    </row>
+    <row r="14" spans="1:12" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1458,21 +1661,24 @@
       <c r="F14" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" s="20" t="s">
         <v>84</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K14" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1490,21 +1696,24 @@
       <c r="F15" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="19" t="s">
         <v>85</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K15" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L15" s="7"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1522,21 +1731,24 @@
       <c r="F16" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" s="20" t="s">
         <v>107</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
       </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K16" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1554,21 +1766,24 @@
       <c r="F17" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="19" t="s">
         <v>108</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="I17" s="15" t="s">
+      <c r="I17" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
       </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K17" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L17" s="7"/>
+    </row>
+    <row r="18" spans="1:12" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1586,21 +1801,24 @@
       <c r="F18" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" s="20" t="s">
         <v>109</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="I18" s="15" t="s">
+      <c r="I18" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K18" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1618,7 +1836,7 @@
       <c r="F19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="G19" s="19" t="s">
         <v>110</v>
       </c>
       <c r="H19" s="7" t="s">
@@ -1630,9 +1848,12 @@
       <c r="J19" s="7">
         <v>1</v>
       </c>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K19" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L19" s="7"/>
+    </row>
+    <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1650,7 +1871,7 @@
       <c r="F20" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="20" t="s">
         <v>111</v>
       </c>
       <c r="H20" s="9" t="s">
@@ -1662,9 +1883,12 @@
       <c r="J20" s="9">
         <v>1</v>
       </c>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K20" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L20" s="9"/>
+    </row>
+    <row r="21" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1682,7 +1906,7 @@
       <c r="F21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="19" t="s">
         <v>112</v>
       </c>
       <c r="H21" s="7" t="s">
@@ -1694,9 +1918,12 @@
       <c r="J21" s="7">
         <v>1</v>
       </c>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K21" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L21" s="7"/>
+    </row>
+    <row r="22" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1714,7 +1941,7 @@
       <c r="F22" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" s="20" t="s">
         <v>90</v>
       </c>
       <c r="H22" s="9" t="s">
@@ -1726,9 +1953,12 @@
       <c r="J22" s="9">
         <v>1</v>
       </c>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K22" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L22" s="9"/>
+    </row>
+    <row r="23" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1746,7 +1976,7 @@
       <c r="F23" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G23" s="8" t="s">
+      <c r="G23" s="19" t="s">
         <v>113</v>
       </c>
       <c r="H23" s="7" t="s">
@@ -1758,9 +1988,12 @@
       <c r="J23" s="7">
         <v>14</v>
       </c>
-      <c r="K23" s="7"/>
-    </row>
-    <row r="24" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K23" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L23" s="7"/>
+    </row>
+    <row r="24" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1778,7 +2011,7 @@
       <c r="F24" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="20" t="s">
         <v>114</v>
       </c>
       <c r="H24" s="9" t="s">
@@ -1790,9 +2023,12 @@
       <c r="J24" s="9">
         <v>2</v>
       </c>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K24" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L24" s="9"/>
+    </row>
+    <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -1810,7 +2046,7 @@
       <c r="F25" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="19" t="s">
         <v>115</v>
       </c>
       <c r="H25" s="7" t="s">
@@ -1822,9 +2058,12 @@
       <c r="J25" s="7">
         <v>1</v>
       </c>
-      <c r="K25" s="7"/>
-    </row>
-    <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K25" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L25" s="7"/>
+    </row>
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -1842,7 +2081,7 @@
       <c r="F26" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="20" t="s">
         <v>116</v>
       </c>
       <c r="H26" s="9" t="s">
@@ -1854,9 +2093,12 @@
       <c r="J26" s="9">
         <v>1</v>
       </c>
-      <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K26" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L26" s="9"/>
+    </row>
+    <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -1874,7 +2116,7 @@
       <c r="F27" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="19" t="s">
         <v>117</v>
       </c>
       <c r="H27" s="7" t="s">
@@ -1886,9 +2128,12 @@
       <c r="J27" s="7">
         <v>1</v>
       </c>
-      <c r="K27" s="7"/>
-    </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K27" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L27" s="7"/>
+    </row>
+    <row r="28" spans="1:12" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -1906,21 +2151,24 @@
       <c r="F28" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" s="20" t="s">
         <v>91</v>
       </c>
       <c r="H28" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="I28" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
       </c>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K28" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -1936,21 +2184,24 @@
       <c r="F29" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="19" t="s">
         <v>118</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="I29" s="15" t="s">
+      <c r="I29" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
       </c>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K29" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L29" s="7"/>
+    </row>
+    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -1968,21 +2219,24 @@
       <c r="F30" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" s="20" t="s">
         <v>119</v>
       </c>
       <c r="H30" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="I30" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
       </c>
-      <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K30" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="1:12" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2000,21 +2254,24 @@
       <c r="F31" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="19" t="s">
         <v>120</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="I31" s="15" t="s">
+      <c r="I31" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
       </c>
-      <c r="K31" s="7"/>
-    </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K31" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L31" s="7"/>
+    </row>
+    <row r="32" spans="1:12" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2030,21 +2287,24 @@
       <c r="F32" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="G32" s="20" t="s">
         <v>121</v>
       </c>
       <c r="H32" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="I32" s="14" t="s">
         <v>167</v>
       </c>
       <c r="J32" s="9">
         <v>2</v>
       </c>
-      <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K32" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2062,7 +2322,7 @@
       <c r="F33" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="19" t="s">
         <v>96</v>
       </c>
       <c r="H33" s="7" t="s">
@@ -2074,9 +2334,12 @@
       <c r="J33" s="7">
         <v>1</v>
       </c>
-      <c r="K33" s="7"/>
-    </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K33" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L33" s="7"/>
+    </row>
+    <row r="34" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2094,10 +2357,10 @@
       <c r="F34" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="G34" s="10" t="s">
+      <c r="G34" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="7" t="s">
         <v>143</v>
       </c>
       <c r="I34" s="10" t="s">
@@ -2106,16 +2369,48 @@
       <c r="J34" s="9">
         <v>1</v>
       </c>
-      <c r="K34" s="9"/>
+      <c r="K34" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L34" s="9"/>
+    </row>
+    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="11">
+        <v>33</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="F35" s="7"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7">
+        <v>1</v>
+      </c>
+      <c r="K35" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="L35" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I1:L1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G1:G1048576">
+  <conditionalFormatting sqref="G1:G34 G36:G1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="K35" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#6 U3 & U5 updated in BOM: Fresh Deliverables remaining.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM-Brendon_STM32-v1.1.xlsx
+++ b/Design_Files/BOM/Client_BOM-Brendon_STM32-v1.1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="174">
   <si>
     <t>#</t>
   </si>
@@ -246,9 +246,6 @@
     <t>IC MCU 32BIT 64KB FLASH 100LQFP</t>
   </si>
   <si>
-    <t>MC14511B Series 3 to 18 Vdc BCD-to-7 Segment Latch/Decoder/Driver - SOIC-16W</t>
-  </si>
-  <si>
     <t>IC 8-BIT TRNSLTR 15KV ESD 20VQFN</t>
   </si>
   <si>
@@ -303,9 +300,6 @@
     <t>LQFP-100</t>
   </si>
   <si>
-    <t>16-SOIC (0.295", 7.50mm Width)</t>
-  </si>
-  <si>
     <t>20-VFQFN Exposed Pad</t>
   </si>
   <si>
@@ -381,9 +375,6 @@
     <t>STM32L071V8T6</t>
   </si>
   <si>
-    <t>MC14511BDWR2G</t>
-  </si>
-  <si>
     <t>TXB0108RGYR</t>
   </si>
   <si>
@@ -541,6 +532,15 @@
   </si>
   <si>
     <t>Through Hole-1.27mm</t>
+  </si>
+  <si>
+    <t>MC14511BDG; Decoder; Driver; Latch; Non-Inverting; 3 - 18 V; 16-Pin SOIC</t>
+  </si>
+  <si>
+    <t>16-SOIC (0.154", 3.90mm Width)</t>
+  </si>
+  <si>
+    <t>MC14511BDG</t>
   </si>
 </sst>
 </file>
@@ -795,9 +795,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -819,82 +816,15 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1204,9 +1134,9 @@
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" style="24" customWidth="1"/>
+    <col min="5" max="5" width="30" style="23" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.5703125" style="21" customWidth="1"/>
+    <col min="7" max="7" width="36.5703125" style="20" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
@@ -1219,14 +1149,14 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="22"/>
+      <c r="E1" s="21"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="18"/>
+      <c r="G1" s="17"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1239,29 +1169,29 @@
       <c r="D2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="22" t="s">
         <v>47</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1280,22 +1210,22 @@
         <v>48</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G3" s="19" t="s">
-        <v>99</v>
+        <v>79</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>97</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J3" s="7">
         <v>19</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L3" s="7"/>
     </row>
@@ -1315,22 +1245,22 @@
         <v>49</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4" s="20" t="s">
-        <v>100</v>
+        <v>79</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>98</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L4" s="9"/>
     </row>
@@ -1350,22 +1280,22 @@
         <v>50</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G5" s="19" t="s">
-        <v>101</v>
+        <v>79</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>99</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L5" s="7"/>
     </row>
@@ -1385,22 +1315,22 @@
         <v>51</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G6" s="20" t="s">
-        <v>102</v>
+        <v>79</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>100</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J6" s="9">
         <v>3</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L6" s="9"/>
     </row>
@@ -1420,22 +1350,22 @@
         <v>52</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>103</v>
+        <v>79</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>101</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J7" s="7">
         <v>4</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L7" s="7"/>
     </row>
@@ -1455,22 +1385,22 @@
         <v>53</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="20" t="s">
-        <v>104</v>
+        <v>80</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>102</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L8" s="9"/>
     </row>
@@ -1481,26 +1411,26 @@
         <v>7</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="8"/>
       <c r="F9" s="7"/>
-      <c r="G9" s="19"/>
+      <c r="G9" s="18"/>
       <c r="H9" s="7"/>
       <c r="I9" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J9" s="15">
         <v>3</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1510,7 +1440,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>22</v>
@@ -1519,22 +1449,22 @@
         <v>54</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="G10" s="20">
+        <v>169</v>
+      </c>
+      <c r="G10" s="19">
         <v>22232021</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J10" s="9">
         <v>4</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L10" s="9"/>
     </row>
@@ -1554,22 +1484,22 @@
         <v>55</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="G11" s="19" t="s">
-        <v>105</v>
+        <v>170</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>103</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L11" s="7"/>
     </row>
@@ -1589,22 +1519,22 @@
         <v>56</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="G12" s="20">
+        <v>169</v>
+      </c>
+      <c r="G12" s="19">
         <v>22232041</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L12" s="9"/>
     </row>
@@ -1624,22 +1554,22 @@
         <v>57</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="G13" s="19" t="s">
-        <v>106</v>
+        <v>82</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>104</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L13" s="7"/>
     </row>
@@ -1659,22 +1589,22 @@
         <v>58</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G14" s="20" t="s">
-        <v>84</v>
+        <v>162</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>83</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L14" s="9"/>
     </row>
@@ -1685,7 +1615,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>27</v>
@@ -1694,22 +1624,22 @@
         <v>59</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G15" s="19" t="s">
-        <v>85</v>
+        <v>162</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>84</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L15" s="7"/>
     </row>
@@ -1729,22 +1659,22 @@
         <v>60</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G16" s="20" t="s">
-        <v>107</v>
+        <v>85</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>105</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L16" s="9"/>
     </row>
@@ -1764,22 +1694,22 @@
         <v>61</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="G17" s="19" t="s">
-        <v>108</v>
+        <v>85</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>106</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L17" s="7"/>
     </row>
@@ -1799,22 +1729,22 @@
         <v>62</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="G18" s="20" t="s">
-        <v>109</v>
+        <v>86</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>107</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L18" s="9"/>
     </row>
@@ -1834,22 +1764,22 @@
         <v>63</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G19" s="19" t="s">
-        <v>110</v>
+        <v>87</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>108</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L19" s="7"/>
     </row>
@@ -1869,22 +1799,22 @@
         <v>64</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="G20" s="20" t="s">
-        <v>111</v>
+        <v>87</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>109</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L20" s="9"/>
     </row>
@@ -1904,22 +1834,22 @@
         <v>65</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>112</v>
+        <v>88</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L21" s="7"/>
     </row>
@@ -1939,22 +1869,22 @@
         <v>66</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="G22" s="20" t="s">
-        <v>90</v>
+        <v>163</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>89</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L22" s="9"/>
     </row>
@@ -1974,22 +1904,22 @@
         <v>67</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>113</v>
+        <v>87</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>111</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J23" s="7">
         <v>14</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L23" s="7"/>
     </row>
@@ -2009,22 +1939,22 @@
         <v>68</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G24" s="20" t="s">
-        <v>114</v>
+        <v>88</v>
+      </c>
+      <c r="G24" s="19" t="s">
+        <v>112</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L24" s="9"/>
     </row>
@@ -2044,22 +1974,22 @@
         <v>69</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G25" s="19" t="s">
-        <v>115</v>
+        <v>87</v>
+      </c>
+      <c r="G25" s="18" t="s">
+        <v>113</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L25" s="7"/>
     </row>
@@ -2079,22 +2009,22 @@
         <v>70</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="G26" s="20" t="s">
-        <v>116</v>
+        <v>87</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>114</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L26" s="9"/>
     </row>
@@ -2114,22 +2044,22 @@
         <v>71</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G27" s="19" t="s">
-        <v>117</v>
+        <v>88</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>115</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L27" s="7"/>
     </row>
@@ -2149,22 +2079,22 @@
         <v>72</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="G28" s="20" t="s">
-        <v>91</v>
+        <v>90</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>90</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L28" s="9"/>
     </row>
@@ -2174,7 +2104,9 @@
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="12"/>
+      <c r="C29" s="13" t="s">
+        <v>12</v>
+      </c>
       <c r="D29" s="7" t="s">
         <v>41</v>
       </c>
@@ -2182,22 +2114,22 @@
         <v>73</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="G29" s="19" t="s">
-        <v>118</v>
+        <v>91</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>116</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L29" s="7"/>
     </row>
@@ -2217,22 +2149,22 @@
         <v>74</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="G30" s="20" t="s">
-        <v>119</v>
+        <v>92</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>117</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L30" s="9"/>
     </row>
@@ -2242,32 +2174,32 @@
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>75</v>
+        <v>171</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="G31" s="19" t="s">
-        <v>120</v>
+        <v>172</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>173</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I31" s="14" t="s">
-        <v>167</v>
+        <v>137</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>173</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L31" s="7"/>
     </row>
@@ -2277,30 +2209,32 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="13"/>
+      <c r="C32" s="13" t="s">
+        <v>12</v>
+      </c>
       <c r="D32" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="G32" s="20" t="s">
-        <v>121</v>
+        <v>93</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>118</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J32" s="9">
         <v>2</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L32" s="9"/>
     </row>
@@ -2317,25 +2251,25 @@
         <v>45</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G33" s="19" t="s">
-        <v>96</v>
+        <v>162</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>94</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L33" s="7"/>
     </row>
@@ -2352,25 +2286,25 @@
         <v>46</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G34" s="20" t="s">
-        <v>97</v>
+        <v>162</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>95</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="L34" s="9"/>
     </row>
@@ -2379,30 +2313,30 @@
         <v>33</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="10" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F35" s="7"/>
-      <c r="G35" s="20"/>
+      <c r="G35" s="19"/>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="7">
         <v>1</v>
       </c>
-      <c r="K35" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="L35" s="17"/>
+      <c r="K35" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="L35" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="G1:G34 G36:G1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G35">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>